<commit_message>
chore : derniers modifications
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_BorminKiril.xlsx
+++ b/Journal-de-Travail_BorminKiril.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\GitHub\165-todo-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFEC4849-CB12-4B13-AB19-F79BD3F2B95D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C34CB61-A8B6-4D4C-B8A0-D91CEFA39D23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33105" yWindow="2385" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="33450" yWindow="2730" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="47">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -179,6 +179,9 @@
   </si>
   <si>
     <t>Remplir le jdt</t>
+  </si>
+  <si>
+    <t>Derniers corrections</t>
   </si>
 </sst>
 </file>
@@ -1189,13 +1192,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>520</c:v>
+                  <c:v>490</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>20</c:v>
+                  <c:v>70</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2044,13 +2047,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.96296296296296291</c:v>
+                  <c:v>0.875</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.7037037037037035E-2</c:v>
+                  <c:v>0.125</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4285,7 +4288,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>9 heures 0 minutes</v>
+        <v>9 heures 20 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4304,11 +4307,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>420</v>
+        <v>440</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>540</v>
+        <v>560</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4602,7 +4605,7 @@
         <v>30</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F16" s="23" t="s">
         <v>40</v>
@@ -4702,15 +4705,23 @@
       <c r="G20" s="39"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="63" t="str">
+      <c r="A21" s="63">
         <f>IF(ISBLANK(B21),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B21))</f>
-        <v/>
-      </c>
-      <c r="B21" s="34"/>
+        <v>21</v>
+      </c>
+      <c r="B21" s="34">
+        <v>46160</v>
+      </c>
       <c r="C21" s="35"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="23"/>
+      <c r="D21" s="36">
+        <v>20</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F21" s="23" t="s">
+        <v>46</v>
+      </c>
       <c r="G21" s="40"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -11020,11 +11031,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>400</v>
+        <v>370</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>520</v>
+        <v>490</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11032,11 +11043,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>8 h 40 min</v>
+        <v>8 h 10 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.96296296296296291</v>
+        <v>0.875</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11094,11 +11105,11 @@
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11106,11 +11117,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>0 h 20 min</v>
+        <v>1 h 10 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>3.7037037037037035E-2</v>
+        <v>0.125</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11166,22 +11177,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>420</v>
+        <v>440</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>540</v>
+        <v>560</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>9 h 00 min</v>
+        <v>9 h 20 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.1</v>
+        <v>0.1037037037037037</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11220,26 +11231,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="62349bcdb43c26c508700efba1cb50b1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e5d6db3f342a25e0e30f4a2965162e1" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11428,10 +11419,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1424D28F-D6A9-45ED-AED5-A0D744400EE5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11454,20 +11476,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1424D28F-D6A9-45ED-AED5-A0D744400EE5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>